<commit_message>
feat: need to move list of figures
</commit_message>
<xml_diff>
--- a/Final/testing/v2_alexnet/v2_alexnet_results.xlsx
+++ b/Final/testing/v2_alexnet/v2_alexnet_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iamkr\Documents\part-4-project\Final\testing\v2_alexnet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6396DDC5-DC67-471A-B2B0-6E16B5998FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78EE6AC4-B247-4EA3-A930-D493F3504D2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="optimised systolic array result" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="97">
   <si>
     <t>Tile</t>
   </si>
@@ -297,6 +297,39 @@
   </si>
   <si>
     <t>Difference from Baseline</t>
+  </si>
+  <si>
+    <t>Fmax</t>
+  </si>
+  <si>
+    <t>Set Up</t>
+  </si>
+  <si>
+    <t>Hold</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>Slow 1100mV 0C</t>
+  </si>
+  <si>
+    <t>289.27 MHz</t>
+  </si>
+  <si>
+    <t>0.308ns</t>
+  </si>
+  <si>
+    <t>6.543ns</t>
+  </si>
+  <si>
+    <t>294.9 MHz</t>
+  </si>
+  <si>
+    <t>0.292 ns</t>
+  </si>
+  <si>
+    <t>6.609 ns</t>
   </si>
 </sst>
 </file>
@@ -373,11 +406,6 @@
   </cellStyles>
   <dxfs count="30">
     <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -423,6 +451,11 @@
     </dxf>
     <dxf>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -786,7 +819,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-NZ"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -911,7 +944,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-NZ"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1619,7 +1652,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FE9EBA62-87A6-48DE-9FD0-115C9888FB6D}" name="Table8" displayName="Table8" ref="L2:M15" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FE9EBA62-87A6-48DE-9FD0-115C9888FB6D}" name="Table8" displayName="Table8" ref="L2:M15" totalsRowShown="0" headerRowDxfId="16">
   <autoFilter ref="L2:M15" xr:uid="{FE9EBA62-87A6-48DE-9FD0-115C9888FB6D}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{153C72B5-F301-4381-83B2-9C6CB91D79D0}" name="Sparsity"/>
@@ -1630,12 +1663,25 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{73C64079-F30E-479D-A80B-7BF29F2E9CAF}" name="Table5" displayName="Table5" ref="A2:C10" totalsRowShown="0" headerRowDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{76781805-1004-4A27-A029-5A4FA5EC8E7C}" name="Table9" displayName="Table9" ref="O2:R4" totalsRowShown="0">
+  <autoFilter ref="O2:R4" xr:uid="{76781805-1004-4A27-A029-5A4FA5EC8E7C}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{09B34F29-6506-4BA4-B9BE-4F4B270D42E6}" name="Model"/>
+    <tableColumn id="2" xr3:uid="{1633A484-8860-42A0-A03D-AC3E692C62B5}" name="Fmax"/>
+    <tableColumn id="3" xr3:uid="{3C85A29F-AEAC-44E4-BB4F-0304819264B7}" name="Set Up"/>
+    <tableColumn id="4" xr3:uid="{E33D93EA-0920-456E-9C1F-DF9488A6661D}" name="Hold"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{73C64079-F30E-479D-A80B-7BF29F2E9CAF}" name="Table5" displayName="Table5" ref="A2:C10" totalsRowShown="0" headerRowDxfId="15">
   <autoFilter ref="A2:C10" xr:uid="{73C64079-F30E-479D-A80B-7BF29F2E9CAF}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{4223D068-5DA5-444E-B53E-3E04385544AC}" name="Size of Matrix A" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{D6124365-E85B-4316-9744-B5FA106748A8}" name="Size of Matrix B" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{8E6C3C48-F7B8-428E-B5FD-3855000F9B12}" name="Latency" dataDxfId="13">
+    <tableColumn id="1" xr3:uid="{4223D068-5DA5-444E-B53E-3E04385544AC}" name="Size of Matrix A" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{D6124365-E85B-4316-9744-B5FA106748A8}" name="Size of Matrix B" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{8E6C3C48-F7B8-428E-B5FD-3855000F9B12}" name="Latency" dataDxfId="12">
       <calculatedColumnFormula>3*8-1</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1643,34 +1689,34 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{3838693E-2926-4C79-A48B-2D9D94DA33FB}" name="Table58" displayName="Table58" ref="G2:H10" totalsRowShown="0" headerRowDxfId="12">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{3838693E-2926-4C79-A48B-2D9D94DA33FB}" name="Table58" displayName="Table58" ref="G2:H10" totalsRowShown="0" headerRowDxfId="11">
   <autoFilter ref="G2:H10" xr:uid="{3838693E-2926-4C79-A48B-2D9D94DA33FB}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{DE127D02-7363-4295-AF36-DDD6DDBD390C}" name="Size of Matrix A and Matrix B" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{DE127D02-7363-4295-AF36-DDD6DDBD390C}" name="Size of Matrix A and Matrix B" dataDxfId="10"/>
     <tableColumn id="3" xr3:uid="{1F86A7D0-C0ED-4BD0-8855-C8E934AD579D}" name="Latency"/>
   </tableColumns>
   <tableStyleInfo name="Table Style 1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B8E41667-AB07-4658-B8AC-6CD371733CB2}" name="Table13" displayName="Table13" ref="A2:I10" totalsRowShown="0" headerRowDxfId="10">
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B8E41667-AB07-4658-B8AC-6CD371733CB2}" name="Table13" displayName="Table13" ref="A2:I10" totalsRowShown="0" headerRowDxfId="9">
   <autoFilter ref="A2:I10" xr:uid="{B8E41667-AB07-4658-B8AC-6CD371733CB2}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D227AF0A-A483-4F2B-A0E7-62312D9D0C8A}" name="Tile"/>
     <tableColumn id="2" xr3:uid="{6A12278B-3584-41AA-BE67-5473F1228243}" name="M"/>
     <tableColumn id="3" xr3:uid="{5020DDA2-0D8A-4E35-BEAF-30F287FD75E9}" name="N"/>
     <tableColumn id="4" xr3:uid="{32BEF9DA-5963-4241-AF0C-B51B609CD406}" name="K"/>
-    <tableColumn id="5" xr3:uid="{7E86E347-49CA-41A8-AEFA-54C42A8E7E80}" name="Output Dimension" dataDxfId="9">
+    <tableColumn id="5" xr3:uid="{7E86E347-49CA-41A8-AEFA-54C42A8E7E80}" name="Output Dimension" dataDxfId="8">
       <calculatedColumnFormula>Table13[[#This Row],[M]]*Table13[[#This Row],[K]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="10" xr3:uid="{309554B3-4463-4DED-AFB0-86EDE0A47AE3}" name="MAC Count (Active PEs)"/>
-    <tableColumn id="6" xr3:uid="{D718F0EC-77E4-469F-8D52-F7CA8782BBE8}" name="Latency (Theory)" dataDxfId="8">
+    <tableColumn id="6" xr3:uid="{D718F0EC-77E4-469F-8D52-F7CA8782BBE8}" name="Latency (Theory)" dataDxfId="7">
       <calculatedColumnFormula>Table13[[#This Row],[M]]+Table13[[#This Row],[N]]+Table13[[#This Row],[K]]-2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{92798A34-7BD8-4D26-B8D7-A549814795F6}" name="Latency (Real)"/>
-    <tableColumn id="8" xr3:uid="{D4FA6A9F-82A1-44DF-9790-64C7064C3DEF}" name="Difference from 3N-2+1" dataDxfId="7">
+    <tableColumn id="8" xr3:uid="{D4FA6A9F-82A1-44DF-9790-64C7064C3DEF}" name="Difference from 3N-2+1" dataDxfId="6">
       <calculatedColumnFormula>23-Table13[[#This Row],[Latency (Real)]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1678,23 +1724,23 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B811506F-69AF-479D-81D3-30BB15DDDBFD}" name="Table134" displayName="Table134" ref="A14:I22" totalsRowShown="0" headerRowDxfId="6">
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B811506F-69AF-479D-81D3-30BB15DDDBFD}" name="Table134" displayName="Table134" ref="A14:I22" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A14:I22" xr:uid="{B811506F-69AF-479D-81D3-30BB15DDDBFD}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{DACD87C0-4923-44EE-9D57-1C4490FF2E04}" name="Tile"/>
     <tableColumn id="2" xr3:uid="{C90B1458-DFBB-4BA7-88F9-708DF57453A0}" name="M"/>
     <tableColumn id="3" xr3:uid="{7E1BAA47-9214-4A68-ACDD-84F7D93D5BAD}" name="N"/>
     <tableColumn id="4" xr3:uid="{193B1B2A-056D-41F1-A31A-35DB3CA612E9}" name="K"/>
-    <tableColumn id="5" xr3:uid="{7A3ECADB-1D1A-44FA-90EB-1828A501A260}" name="Output Dimension" dataDxfId="5">
+    <tableColumn id="5" xr3:uid="{7A3ECADB-1D1A-44FA-90EB-1828A501A260}" name="Output Dimension" dataDxfId="4">
       <calculatedColumnFormula>Table134[[#This Row],[M]]*Table134[[#This Row],[K]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="10" xr3:uid="{17395CC5-C66A-45BB-AF44-85F63C798FE8}" name="MAC Count (Active PEs)"/>
-    <tableColumn id="6" xr3:uid="{F344959C-0D04-4AF5-B2C4-FF7C3F674B16}" name="Latency (Theory)" dataDxfId="4">
+    <tableColumn id="6" xr3:uid="{F344959C-0D04-4AF5-B2C4-FF7C3F674B16}" name="Latency (Theory)" dataDxfId="3">
       <calculatedColumnFormula>Table134[[#This Row],[M]]+Table134[[#This Row],[N]]+Table134[[#This Row],[K]]-2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{7EEC49AA-4FC8-4A99-9663-A8EEB2AAD5F8}" name="Latency (Real)"/>
-    <tableColumn id="8" xr3:uid="{B71F4CFD-5FC5-4951-83D9-6674EB7FB889}" name="Difference from 3N-2+1" dataDxfId="3">
+    <tableColumn id="8" xr3:uid="{B71F4CFD-5FC5-4951-83D9-6674EB7FB889}" name="Difference from 3N-2+1" dataDxfId="2">
       <calculatedColumnFormula>23-Table134[[#This Row],[Latency (Real)]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1702,7 +1748,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BA1FDD35-9C8D-43D3-A42C-5D9448260A9A}" name="Table1" displayName="Table1" ref="A2:H10" totalsRowShown="0">
   <autoFilter ref="A2:H10" xr:uid="{BA1FDD35-9C8D-43D3-A42C-5D9448260A9A}"/>
   <tableColumns count="8">
@@ -1710,14 +1756,14 @@
     <tableColumn id="2" xr3:uid="{66D560B9-2DA7-4986-B3DE-CDA502776AC3}" name="M"/>
     <tableColumn id="3" xr3:uid="{5141C682-632F-43C2-8191-BB3609DB4DA8}" name="N"/>
     <tableColumn id="4" xr3:uid="{A9660E6C-180E-485D-A7EB-A8BFCE0C1D97}" name="K"/>
-    <tableColumn id="5" xr3:uid="{34B7FFF0-3EF6-4BA4-A5AB-1660E75007C8}" name="Output Dimension (MAC Count)" dataDxfId="2">
+    <tableColumn id="5" xr3:uid="{34B7FFF0-3EF6-4BA4-A5AB-1660E75007C8}" name="Output Dimension (MAC Count)" dataDxfId="1">
       <calculatedColumnFormula>4*8</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{3CE6D932-CF3F-4780-8775-A3AC543F142B}" name="Latency">
       <calculatedColumnFormula>Table1[[#This Row],[M]]+Table1[[#This Row],[N]]+Table1[[#This Row],[K]]-2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{3D0DE0B8-37A2-4603-B02E-4FE79DF8244C}" name="Latency (Real)"/>
-    <tableColumn id="8" xr3:uid="{78C59BA1-4582-42E9-8A9A-782701EF4A8A}" name="Difference from 3N-2+1" dataDxfId="1">
+    <tableColumn id="8" xr3:uid="{78C59BA1-4582-42E9-8A9A-782701EF4A8A}" name="Difference from 3N-2+1" dataDxfId="0">
       <calculatedColumnFormula>23-Table1[[#This Row],[Latency (Real)]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1988,7 +2034,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32EAF263-E46A-4974-93A7-B91CE9F0B8F1}">
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:R15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
@@ -2002,9 +2048,12 @@
     <col min="10" max="10" width="25.85546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="24.7109375" customWidth="1"/>
+    <col min="15" max="15" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>84</v>
       </c>
@@ -2023,7 +2072,7 @@
       </c>
       <c r="M1" s="7"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>55</v>
       </c>
@@ -2057,8 +2106,20 @@
       <c r="M2" s="1" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O2" t="s">
+        <v>89</v>
+      </c>
+      <c r="P2" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>87</v>
+      </c>
+      <c r="R2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>0</v>
       </c>
@@ -2093,8 +2154,20 @@
       <c r="M3">
         <v>23</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P3" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>93</v>
+      </c>
+      <c r="R3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -2129,8 +2202,20 @@
       <c r="M4">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O4" t="s">
+        <v>90</v>
+      </c>
+      <c r="P4" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>96</v>
+      </c>
+      <c r="R4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2</v>
       </c>
@@ -2166,7 +2251,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>3</v>
       </c>
@@ -2202,7 +2287,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>4</v>
       </c>
@@ -2238,7 +2323,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>5</v>
       </c>
@@ -2274,7 +2359,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>6</v>
       </c>
@@ -2310,7 +2395,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>7</v>
       </c>
@@ -2346,7 +2431,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>8</v>
       </c>
@@ -2382,7 +2467,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="L12">
         <v>80</v>
       </c>
@@ -2390,7 +2475,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="L13">
         <v>85</v>
       </c>
@@ -2398,7 +2483,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="L14">
         <v>90</v>
       </c>
@@ -2406,7 +2491,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="L15">
         <v>95</v>
       </c>
@@ -2423,10 +2508,11 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
-  <tableParts count="3">
+  <tableParts count="4">
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>